<commit_message>
Require a manufacturer on a new product
Identity is name plus manufacturer, so a product registered without one
leaves nothing to tell it apart from the same name made by someone
else. The blank is what lets a later row merge into it, and once stock
and prices are in, the merge has no undo.

Required now in ProductService as well as the import, so the rule holds
whichever way a product arrives. A row that only updates an existing
product may still leave it empty: the second batch row of a product
carries nothing but the name, and requiring it there would reject a
sheet filled in exactly as the instructions say.

Products registered before this carry no manufacturer until someone
edits them, and the edit screen asks for one when they do. The survey
sheet marks the column required and says why.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/templates/initial-stock-survey.xlsx
+++ b/docs/templates/initial-stock-survey.xlsx
@@ -172,7 +172,10 @@
     <x:t>2. Columns are in the same order as the Add Product screen: identification → price → loose units → barcode → source → antibiotic → batch.</x:t>
   </x:si>
   <x:si>
-    <x:t>3. Required: product_name, dosage_form, unit, selling_price. generic_name is required for medicines — for bandages, tubes, masks choose dosage_form = Other and leave generic_name empty.</x:t>
+    <x:t>3. Required: product_name, manufacturer, dosage_form, unit, selling_price. generic_name is required for medicines — for bandages, tubes, masks choose dosage_form = Other and leave generic_name empty.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>3b. manufacturer decides which product a row is. Two makers of the same name are two separate products, so fill it in even when the name looks unique.</x:t>
   </x:si>
   <x:si>
     <x:t>4. dosage_form and unit are dropdowns — click the cell, then the ▼. Do not type your own spelling; the import checks the value.</x:t>
@@ -286,7 +289,7 @@
     <x:t>8801234567890</x:t>
   </x:si>
   <x:si>
-    <x:t>Manufacturer</x:t>
+    <x:t>Who made it. Two makers of one name = two products</x:t>
   </x:si>
   <x:si>
     <x:t>Sanofi</x:t>
@@ -835,7 +838,7 @@
       <x:c r="L1" s="2" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="M1" s="2" t="s">
+      <x:c r="M1" s="1" t="s">
         <x:v>39</x:v>
       </x:c>
       <x:c r="N1" s="2" t="s">
@@ -23023,7 +23026,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:A14"/>
+  <x:dimension ref="A1:A15"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="130.710625" style="4" customWidth="1"/>
@@ -23091,12 +23094,17 @@
     </x:row>
     <x:row r="13" spans="1:1">
       <x:c r="A13" s="4" t="s">
+        <x:v>59</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" spans="1:1">
+      <x:c r="A14" s="4" t="s">
         <x:v>48</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" spans="1:1">
-      <x:c r="A14" s="4" t="s">
-        <x:v>59</x:v>
+    <x:row r="15" spans="1:1">
+      <x:c r="A15" s="4" t="s">
+        <x:v>60</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -23124,16 +23132,16 @@
   <x:sheetData>
     <x:row r="1" spans="1:4" s="6" customFormat="1">
       <x:c r="A1" s="6" t="s">
-        <x:v>60</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="B1" s="6" t="s">
-        <x:v>61</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C1" s="6" t="s">
-        <x:v>62</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="D1" s="6" t="s">
-        <x:v>63</x:v>
+        <x:v>64</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:4">
@@ -23141,13 +23149,13 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="C2" s="7" t="s">
-        <x:v>65</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="D2" s="3" t="s">
-        <x:v>66</x:v>
+        <x:v>67</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:4">
@@ -23155,13 +23163,13 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="C3" s="7" t="s">
-        <x:v>68</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="D3" s="3" t="s">
-        <x:v>69</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:4">
@@ -23169,13 +23177,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>70</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="D4" s="3" t="s">
-        <x:v>72</x:v>
+        <x:v>73</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:4">
@@ -23183,10 +23191,10 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>73</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="C5" s="7" t="s">
-        <x:v>65</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="D5" s="3" t="s">
         <x:v>1</x:v>
@@ -23197,10 +23205,10 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="C6" s="7" t="s">
-        <x:v>65</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="D6" s="3" t="s">
         <x:v>1</x:v>
@@ -23211,13 +23219,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
-        <x:v>75</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C7" s="7" t="s">
-        <x:v>65</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="D7" s="3" t="s">
-        <x:v>76</x:v>
+        <x:v>77</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:4">
@@ -23225,13 +23233,13 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
-        <x:v>77</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="C8" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="D8" s="3" t="s">
-        <x:v>78</x:v>
+        <x:v>79</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:4">
@@ -23239,13 +23247,13 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="B9" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C9" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="D9" s="3" t="s">
-        <x:v>80</x:v>
+        <x:v>81</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:4">
@@ -23253,10 +23261,10 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="B10" s="0" t="s">
-        <x:v>81</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="C10" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="D10" s="3" t="s">
         <x:v>23</x:v>
@@ -23267,13 +23275,13 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="B11" s="0" t="s">
-        <x:v>82</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="C11" s="0" t="s">
-        <x:v>83</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="D11" s="3" t="s">
-        <x:v>84</x:v>
+        <x:v>85</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:4">
@@ -23281,13 +23289,13 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="B12" s="0" t="s">
-        <x:v>85</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="C12" s="0" t="s">
-        <x:v>83</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="D12" s="3" t="s">
-        <x:v>86</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:4">
@@ -23295,13 +23303,13 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="B13" s="0" t="s">
-        <x:v>87</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="C13" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="D13" s="3" t="s">
-        <x:v>88</x:v>
+        <x:v>89</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:4">
@@ -23309,13 +23317,13 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="B14" s="0" t="s">
-        <x:v>89</x:v>
+        <x:v>90</x:v>
       </x:c>
-      <x:c r="C14" s="0" t="s">
-        <x:v>71</x:v>
+      <x:c r="C14" s="7" t="s">
+        <x:v>66</x:v>
       </x:c>
       <x:c r="D14" s="3" t="s">
-        <x:v>90</x:v>
+        <x:v>91</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:4">
@@ -23323,13 +23331,13 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="B15" s="0" t="s">
-        <x:v>91</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="C15" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="D15" s="3" t="s">
-        <x:v>92</x:v>
+        <x:v>93</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:4">
@@ -23337,13 +23345,13 @@
         <x:v>41</x:v>
       </x:c>
       <x:c r="B16" s="0" t="s">
-        <x:v>93</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="C16" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="D16" s="3" t="s">
-        <x:v>94</x:v>
+        <x:v>95</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:4">
@@ -23351,10 +23359,10 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="B17" s="0" t="s">
-        <x:v>95</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="C17" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="D17" s="3" t="s">
         <x:v>26</x:v>
@@ -23365,13 +23373,13 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="B18" s="0" t="s">
-        <x:v>96</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="C18" s="0" t="s">
-        <x:v>97</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="D18" s="3" t="s">
-        <x:v>98</x:v>
+        <x:v>99</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:4">
@@ -23379,13 +23387,13 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="B19" s="0" t="s">
-        <x:v>99</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="C19" s="0" t="s">
-        <x:v>97</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="D19" s="3" t="s">
-        <x:v>100</x:v>
+        <x:v>101</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:4">
@@ -23393,13 +23401,13 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="B20" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="C20" s="7" t="s">
-        <x:v>102</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="D20" s="3" t="s">
-        <x:v>103</x:v>
+        <x:v>104</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:4">
@@ -23407,10 +23415,10 @@
         <x:v>46</x:v>
       </x:c>
       <x:c r="B21" s="0" t="s">
-        <x:v>104</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="C21" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="D21" s="3" t="s">
         <x:v>48</x:v>

</xml_diff>